<commit_message>
Add baseline test numbers
</commit_message>
<xml_diff>
--- a/data/pepfar_modalities.xlsx
+++ b/data/pepfar_modalities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{707DAA9B-B2E9-7A49-B525-1282AFD9A1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4858EB9-E700-8544-9C1A-FF8E259CDCB7}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="8_{707DAA9B-B2E9-7A49-B525-1282AFD9A1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A23531B9-275D-9441-83DE-DD26F492C320}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{10B07BF5-BE7F-0742-9720-A8DB39804C05}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
   <si>
     <t>TBClinic</t>
   </si>
@@ -178,13 +178,37 @@
   </si>
   <si>
     <t>Modality</t>
+  </si>
+  <si>
+    <t>test_facility_general</t>
+  </si>
+  <si>
+    <t>test_community</t>
+  </si>
+  <si>
+    <t>test_index</t>
+  </si>
+  <si>
+    <t>anc_hiv_testing</t>
+  </si>
+  <si>
+    <t>pnc_hiv_testing</t>
+  </si>
+  <si>
+    <t>test_kpsti</t>
+  </si>
+  <si>
+    <t>test_network</t>
+  </si>
+  <si>
+    <t>other</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -322,6 +346,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -675,10 +706,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1058,6 +1090,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1072,8 +1105,8 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
-        <v>42</v>
+      <c r="B2" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="F2" s="1"/>
     </row>
@@ -1081,249 +1114,264 @@
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>42</v>
+      <c r="B3" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
-        <v>39</v>
+      <c r="B4" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
-        <v>39</v>
+      <c r="B5" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
-        <v>40</v>
+      <c r="B6" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
-        <v>40</v>
+      <c r="B7" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>42</v>
+      <c r="B8" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>33</v>
       </c>
-      <c r="B9" t="s">
-        <v>35</v>
+      <c r="B9" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
-        <v>42</v>
+      <c r="B10" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B11" t="s">
-        <v>35</v>
+      <c r="B11" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
-        <v>39</v>
+      <c r="B12" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
-      <c r="B13" t="s">
-        <v>39</v>
+      <c r="B13" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>18</v>
       </c>
+      <c r="B14" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>4</v>
       </c>
-      <c r="B15" t="s">
-        <v>42</v>
+      <c r="B15" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
-        <v>42</v>
+      <c r="B16" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>28</v>
       </c>
+      <c r="B17" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>21</v>
       </c>
+      <c r="B18" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>30</v>
       </c>
-      <c r="B19" t="s">
-        <v>42</v>
+      <c r="B19" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="2"/>
+      <c r="B20" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>5</v>
       </c>
-      <c r="B21" t="s">
-        <v>35</v>
+      <c r="B21" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>27</v>
       </c>
-      <c r="B22" t="s">
-        <v>36</v>
+      <c r="B22" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>26</v>
       </c>
-      <c r="B23" t="s">
-        <v>35</v>
+      <c r="B23" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>1</v>
       </c>
-      <c r="B24" t="s">
-        <v>36</v>
+      <c r="B24" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>6</v>
       </c>
-      <c r="B25" t="s">
-        <v>41</v>
+      <c r="B25" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>20</v>
       </c>
-      <c r="B26" t="s">
-        <v>40</v>
+      <c r="B26" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>13</v>
       </c>
-      <c r="B27" t="s">
-        <v>40</v>
+      <c r="B27" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>2</v>
       </c>
-      <c r="B28" t="s">
-        <v>41</v>
+      <c r="B28" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>0</v>
       </c>
-      <c r="B29" t="s">
-        <v>42</v>
+      <c r="B29" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="2"/>
+      <c r="B30" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>42</v>
+      <c r="B31" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>42</v>
+      <c r="B32" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="2"/>
+      <c r="B33" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>42</v>
+      <c r="B34" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>42</v>
+      <c r="B35" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>